<commit_message>
correct typo in glass properties
</commit_message>
<xml_diff>
--- a/cubes/data/materials/windows.xlsx
+++ b/cubes/data/materials/windows.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/elizabeth-homes/src/cubes/data/materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/CUBES/cubes/data/materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDF4B3C-5750-4045-9FC3-B169DCBF4D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EC8EE5-5915-5241-A23D-DFA443C88EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4920" yWindow="-21760" windowWidth="25200" windowHeight="18380" xr2:uid="{47704123-5C42-9841-98FC-8623E63A368D}"/>
   </bookViews>
@@ -483,6 +483,9 @@
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
@@ -744,10 +747,10 @@
         <v>0.85</v>
       </c>
       <c r="I8">
-        <v>0.56000000000000005</v>
+        <v>5.6000000000000001E-2</v>
       </c>
       <c r="J8">
-        <v>0.79</v>
+        <v>7.9000000000000001E-2</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -788,10 +791,10 @@
         <v>0.85</v>
       </c>
       <c r="I9">
-        <v>0.79</v>
+        <v>7.9000000000000001E-2</v>
       </c>
       <c r="J9">
-        <v>0.56000000000000005</v>
+        <v>5.6000000000000001E-2</v>
       </c>
       <c r="K9">
         <v>0</v>

</xml_diff>